<commit_message>
Explain every indicator (what / why / impact, EN+AR), EGX30 + EGX70, explain mode, period labels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/manual/manual_inputs.xlsx
+++ b/data/manual/manual_inputs.xlsx
@@ -63,6 +63,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cpi_med_products_yoy" sheetId="54" state="visible" r:id="rId54"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="drug_shortages" sheetId="55" state="visible" r:id="rId55"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pharma_market" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="egx70" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -894,7 +895,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -996,7 +996,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1098,7 +1097,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1200,7 +1198,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1439,9 +1436,6 @@
           <t>موديز ترفع تصنيف مصر درجة مع نظرة إيجابية</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>confirmed</t>
@@ -1484,9 +1478,6 @@
           <t>فيتش تثبت تصنيف مصر مع نظرة مستقرة</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>confirmed</t>
@@ -1502,7 +1493,6 @@
           <t>https://en.amwalalghad.com/fitch-affirms-egypts-b-rating-with-stable-outlook/</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1525,9 +1515,6 @@
           <t>ستاندرد آند بورز تثبت تصنيف مصر مع نظرة مستقرة</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>reported</t>
@@ -1570,9 +1557,6 @@
           <t>صندوق النقد يخلص المراجعتين الخامسة والسادسة</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>confirmed</t>
@@ -1615,9 +1599,6 @@
           <t>صندوق النقد يخلص المراجعة السابعة ويصرف شريحة جديدة</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>reported</t>
@@ -1660,9 +1641,6 @@
           <t>لجنة تسعير الوقود تثبت الأسعار لحد آخر ديسمبر</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>confirmed</t>
@@ -1705,9 +1683,6 @@
           <t>هيئة الدواء تصدر قرار تسعير جديد</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>reported</t>
@@ -2253,7 +2228,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2501,7 +2475,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2972,7 +2945,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3013,7 +2985,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3054,7 +3025,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3095,7 +3065,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3136,7 +3105,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3177,7 +3145,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3218,7 +3185,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3259,7 +3225,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3300,7 +3265,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3341,7 +3305,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3382,7 +3345,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3423,7 +3385,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3554,7 +3515,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3595,7 +3555,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3636,7 +3595,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3677,7 +3635,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3718,7 +3675,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3804,7 +3760,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3845,7 +3800,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5229,7 +5183,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5331,7 +5284,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5433,7 +5385,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5535,7 +5486,6 @@
           <t>secondary</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6150,6 +6100,62 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>obs_date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>source_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>source_date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>quality_flag</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>